<commit_message>
release 1.0.0: reorg package sim_v1/sim_v2/catboost, api web, pipeline yaml
</commit_message>
<xml_diff>
--- a/accor/data/eval_compare_loo.xlsx
+++ b/accor/data/eval_compare_loo.xlsx
@@ -10,6 +10,7 @@
     <sheet name="metrics" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="detail_sim_v2" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="detail_ia_xgboost" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="detail_ia_dense" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -731,12 +732,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>sim_v1</t>
+          <t>ia_dense</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>regles_excel</t>
+          <t>NN</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -745,38 +746,134 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2968.26</v>
-      </c>
-      <c r="E11" t="inlineStr"/>
+        <v>3339.448278060154</v>
+      </c>
+      <c r="E11" t="n">
+        <v>6521.620259621252</v>
+      </c>
       <c r="F11" t="n">
-        <v>188.7</v>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+        <v>63.84081673830645</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-2493.567139667297</v>
+      </c>
+      <c r="H11" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>ia_dense</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NN</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>montant_marge_par_mois</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1920.175739030659</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3515.248200422094</v>
+      </c>
+      <c r="F12" t="n">
+        <v>90.04301518817024</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-1585.205188308591</v>
+      </c>
+      <c r="H12" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ia_dense</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NN</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>montant_marge_selon_coef_par_mois</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1980.981814900256</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3297.525385184598</v>
+      </c>
+      <c r="F13" t="n">
+        <v>94.52090043406284</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-669.079442467605</v>
+      </c>
+      <c r="H13" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>sim_v1</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>regles_excel</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>montant_ventes_par_mois</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>2968.26</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="n">
+        <v>188.7</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>sim_v1</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>regles_excel</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
         <is>
           <t>montant_marge_par_mois</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D15" t="n">
         <v>2684.42</v>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2497,4 +2594,492 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>modele</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>hotel_code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>solution</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>solution_vue_en_apprentissage</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>montant_ventes_par_mois_reel</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>montant_ventes_par_mois_predit</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>montant_ventes_par_mois_erreur</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>montant_ventes_par_mois_erreur_absolue</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>montant_marge_par_mois_reel</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>montant_marge_par_mois_predit</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>montant_marge_par_mois_erreur</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>montant_marge_par_mois_erreur_absolue</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>montant_marge_selon_coef_par_mois_reel</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>montant_marge_selon_coef_par_mois_predit</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>montant_marge_selon_coef_par_mois_erreur</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>montant_marge_selon_coef_par_mois_erreur_absolue</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ia_dense</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>H0373</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>connected</t>
+        </is>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>3432.306971428518</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2871.049560546875</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-561.257410881643</v>
+      </c>
+      <c r="H2" t="n">
+        <v>561.257410881643</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2214.074874999865</v>
+      </c>
+      <c r="J2" t="n">
+        <v>489.878173828125</v>
+      </c>
+      <c r="K2" t="n">
+        <v>-1724.19670117174</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1724.19670117174</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1977.989434346401</v>
+      </c>
+      <c r="N2" t="n">
+        <v>2996.45947265625</v>
+      </c>
+      <c r="O2" t="n">
+        <v>1018.470038309849</v>
+      </c>
+      <c r="P2" t="n">
+        <v>1018.470038309849</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ia_dense</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>H2075</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>simply</t>
+        </is>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>570.2660606060817</v>
+      </c>
+      <c r="F3" t="n">
+        <v>101.807373046875</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-468.4586875592067</v>
+      </c>
+      <c r="H3" t="n">
+        <v>468.4586875592067</v>
+      </c>
+      <c r="I3" t="n">
+        <v>233.321212121201</v>
+      </c>
+      <c r="J3" t="n">
+        <v>588.7568359375</v>
+      </c>
+      <c r="K3" t="n">
+        <v>355.435623816299</v>
+      </c>
+      <c r="L3" t="n">
+        <v>355.435623816299</v>
+      </c>
+      <c r="M3" t="n">
+        <v>248.7434418642236</v>
+      </c>
+      <c r="N3" t="n">
+        <v>555.0455322265625</v>
+      </c>
+      <c r="O3" t="n">
+        <v>306.3020903623388</v>
+      </c>
+      <c r="P3" t="n">
+        <v>306.3020903623388</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ia_dense</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>H3546</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>connected</t>
+        </is>
+      </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>17096.63041667935</v>
+      </c>
+      <c r="F4" t="n">
+        <v>178.13134765625</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-16918.4990690231</v>
+      </c>
+      <c r="H4" t="n">
+        <v>16918.4990690231</v>
+      </c>
+      <c r="I4" t="n">
+        <v>9167.626249997114</v>
+      </c>
+      <c r="J4" t="n">
+        <v>113.7787475585938</v>
+      </c>
+      <c r="K4" t="n">
+        <v>-9053.847502438521</v>
+      </c>
+      <c r="L4" t="n">
+        <v>9053.847502438521</v>
+      </c>
+      <c r="M4" t="n">
+        <v>8864.534661573482</v>
+      </c>
+      <c r="N4" t="n">
+        <v>564.3300170898438</v>
+      </c>
+      <c r="O4" t="n">
+        <v>-8300.204644483638</v>
+      </c>
+      <c r="P4" t="n">
+        <v>8300.204644483638</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ia_dense</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>H5586</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>connected</t>
+        </is>
+      </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2960.583984375</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2960.583984375</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2960.583984375</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>816.9613037109375</v>
+      </c>
+      <c r="K5" t="n">
+        <v>816.9613037109375</v>
+      </c>
+      <c r="L5" t="n">
+        <v>816.9613037109375</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>2002.995361328125</v>
+      </c>
+      <c r="O5" t="n">
+        <v>2002.995361328125</v>
+      </c>
+      <c r="P5" t="n">
+        <v>2002.995361328125</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ia_dense</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>H6188</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>liberty</t>
+        </is>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1438.426056822751</v>
+      </c>
+      <c r="F6" t="n">
+        <v>392.44140625</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-1045.984650572751</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1045.984650572751</v>
+      </c>
+      <c r="I6" t="n">
+        <v>750.5261190476397</v>
+      </c>
+      <c r="J6" t="n">
+        <v>361.8033447265625</v>
+      </c>
+      <c r="K6" t="n">
+        <v>-388.7227743210772</v>
+      </c>
+      <c r="L6" t="n">
+        <v>388.7227743210772</v>
+      </c>
+      <c r="M6" t="n">
+        <v>795.1738730737154</v>
+      </c>
+      <c r="N6" t="n">
+        <v>364.607177734375</v>
+      </c>
+      <c r="O6" t="n">
+        <v>-430.5666953393404</v>
+      </c>
+      <c r="P6" t="n">
+        <v>430.5666953393404</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ia_dense</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HB5I0</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>liberty</t>
+        </is>
+      </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1766.508730769235</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1257.544677734375</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-508.9640530348597</v>
+      </c>
+      <c r="H7" t="n">
+        <v>508.9640530348597</v>
+      </c>
+      <c r="I7" t="n">
+        <v>974.3293076923151</v>
+      </c>
+      <c r="J7" t="n">
+        <v>394.6619873046875</v>
+      </c>
+      <c r="K7" t="n">
+        <v>-579.6673203876276</v>
+      </c>
+      <c r="L7" t="n">
+        <v>579.6673203876276</v>
+      </c>
+      <c r="M7" t="n">
+        <v>815.1594794547862</v>
+      </c>
+      <c r="N7" t="n">
+        <v>2079.05029296875</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1263.890813513964</v>
+      </c>
+      <c r="P7" t="n">
+        <v>1263.890813513964</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ia_dense</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HB6A3</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>simply</t>
+        </is>
+      </c>
+      <c r="D8" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1085.428421052641</v>
+      </c>
+      <c r="F8" t="n">
+        <v>173.038330078125</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-912.3900909745157</v>
+      </c>
+      <c r="H8" t="n">
+        <v>912.3900909745157</v>
+      </c>
+      <c r="I8" t="n">
+        <v>522.3989473684123</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>-522.3989473684123</v>
+      </c>
+      <c r="L8" t="n">
+        <v>522.3989473684123</v>
+      </c>
+      <c r="M8" t="n">
+        <v>607.1911078395337</v>
+      </c>
+      <c r="N8" t="n">
+        <v>62.748046875</v>
+      </c>
+      <c r="O8" t="n">
+        <v>-544.4430609645337</v>
+      </c>
+      <c r="P8" t="n">
+        <v>544.4430609645337</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>